<commit_message>
Fix unit inconsistency in NDI rows of Nitta valuation sheet
NDI売上 / NDI純利益 だけ億円単位で記載していたため、同列の持分法利益(百万円)と
数値比較したときに「利益>売上」に見える不整合が発生していた。

修正: NDI関連の3行(NDI売上、NDI純利益)を百万円に統一。
- NDI売上 FY3/26: 327億 → 32,700百万円
- NDI純利益 FY3/26: 90億 → 9,018百万円
- NDI持分法利益 FY3/26: 4,509百万円 = NDI純利益 9,018 × 出資比率50%
- NDI純利益率 = 9,018 / 32,700 = 27.6% (CMPパッド高マージン消耗材として妥当)
</commit_message>
<xml_diff>
--- a/outputs/5186-nitta-valuation.xlsx
+++ b/outputs/5186-nitta-valuation.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="5186_nitta_valuation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5186_nitta_valuation" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -249,14 +249,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -280,7 +280,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -304,7 +304,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -328,7 +328,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -352,7 +352,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -382,7 +382,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -390,7 +390,7 @@
             <symbol val="circle"/>
             <size val="7"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -414,8 +414,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -441,8 +441,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -467,8 +467,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -495,14 +495,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -526,7 +526,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -550,7 +550,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -578,8 +578,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -605,8 +605,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -632,14 +632,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -663,7 +663,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -687,7 +687,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -711,7 +711,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -739,8 +739,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -766,8 +766,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -793,7 +793,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -808,9 +808,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -830,9 +830,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -852,9 +852,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2229,26 +2229,26 @@
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t>NDI売上 (CY、億円)</t>
+          <t>NDI売上 (CY、百万円)</t>
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>260</v>
+        <v>26000</v>
       </c>
       <c r="C46" s="13" t="n">
-        <v>280</v>
+        <v>28000</v>
       </c>
       <c r="D46" s="13" t="n">
-        <v>300</v>
+        <v>30000</v>
       </c>
       <c r="E46" s="13" t="n">
-        <v>327</v>
+        <v>32700</v>
       </c>
       <c r="F46" s="13" t="n">
-        <v>360</v>
+        <v>36000</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>410</v>
+        <v>41000</v>
       </c>
       <c r="H46" s="14" t="inlineStr">
         <is>
@@ -2426,27 +2426,27 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>NDI純利益(推計, 億円)</t>
+          <t>NDI純利益(推計, 百万円)</t>
         </is>
       </c>
       <c r="B53" s="7" t="n"/>
       <c r="C53" s="7" t="n"/>
       <c r="D53" s="7" t="n">
-        <v>80</v>
+        <v>8010</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>90</v>
+        <v>9018</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>104</v>
+        <v>10400</v>
       </c>
       <c r="G53" s="7" t="n">
-        <v>112</v>
+        <v>11200</v>
       </c>
       <c r="H53" s="4" t="inlineStr"/>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>NDI持分法利益 ÷ 出資比率50% で逆算 (FY3/26: 4,509百万 ÷ 0.50 = 90億)。NDI営業利益率と税率の整合チェック用</t>
+          <t>NDI持分法利益 ÷ 出資比率50% で逆算 (FY3/26: 4,509百万 ÷ 0.50 = 9,018百万 = 90億)。NDI純利益率 ≒ 9,018/32,700 = 27.6%</t>
         </is>
       </c>
     </row>

</xml_diff>